<commit_message>
fix: update sce compartment information
</commit_message>
<xml_diff>
--- a/data/sce_compartment_curation/mitochondrial_suborganelle.xlsx
+++ b/data/sce_compartment_curation/mitochondrial_suborganelle.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xluhon/Documents/GitHub/large_scale_yeast_proteomics_analysis/data/sce_compartment_curation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E750310-8D5A-1542-B19F-8072B094BBC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D28D20A1-2D55-CC4E-8A20-3C524B26E2EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5780" yWindow="4260" windowWidth="29480" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5780" yWindow="4260" windowWidth="29480" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Supplementary Data 5" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Supplementary Data 5'!$A$1:$Q$1</definedName>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4864" uniqueCount="2848">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4865" uniqueCount="2849">
   <si>
     <t>Gene</t>
   </si>
@@ -8722,6 +8723,9 @@
   <si>
     <t>gene</t>
   </si>
+  <si>
+    <t>https://www.nature.com/articles/s41467-017-00359-0#Sec24 Landscape of submitochondrial protein distribution</t>
+  </si>
 </sst>
 </file>
 
@@ -8730,7 +8734,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -8800,6 +8804,13 @@
       <b/>
       <i/>
       <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -9082,13 +9093,14 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -9237,8 +9249,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="4"/>
   </cellXfs>
-  <cellStyles count="4">
+  <cellStyles count="5">
+    <cellStyle name="Hyperlink" xfId="4" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Per cent" xfId="1" builtinId="5"/>
     <cellStyle name="Prozent 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
@@ -53858,4 +53872,22 @@
     </ext>
   </extLst>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5FE63F4-B0E6-4249-85FE-1D9F1E3BB60F}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1" s="50" t="s">
+        <v>2848</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A1" r:id="rId1" location="Sec24 Landscape of submitochondrial protein distribution" xr:uid="{9D92CF22-7BDB-CE42-B6E9-DBFBD7470F96}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>